<commit_message>
Added SEIR actions and events into the simulation.
</commit_message>
<xml_diff>
--- a/map/city/routes.xlsx
+++ b/map/city/routes.xlsx
@@ -1,37 +1,60 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Unida\Documents\VSC\Python\EpidemicSimulation\map\city\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C87B59-CBA2-485D-8E76-543DEB4449BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="24300" yWindow="588" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Node 1</t>
+  </si>
+  <si>
+    <t>Node 2</t>
+  </si>
+  <si>
+    <t>Interval</t>
+  </si>
+  <si>
+    <t>Peak Interval</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +69,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,248 +393,414 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Node 1</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Node 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>23</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2">
         <v>535</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="C2">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>137</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3">
         <v>224</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="C3">
+        <v>6</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>109</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4">
         <v>169</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="C4">
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>25</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5">
         <v>535</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>28</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6">
         <v>532</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="C6">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>336</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7">
         <v>303</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>46</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8">
         <v>111</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>365</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9">
         <v>303</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
+      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>137</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10">
         <v>72</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>28</v>
       </c>
-      <c r="B11" t="n">
+      <c r="B11">
         <v>532</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
+      <c r="C11">
+        <v>6</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>491</v>
       </c>
-      <c r="B12" t="n">
+      <c r="B12">
         <v>365</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
+      <c r="C12">
+        <v>6</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>530</v>
       </c>
-      <c r="B13" t="n">
+      <c r="B13">
         <v>537</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
+      <c r="C13">
+        <v>6</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>191</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14">
         <v>285</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
+      <c r="C14">
+        <v>6</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>233</v>
       </c>
-      <c r="B15" t="n">
+      <c r="B15">
         <v>537</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
+      <c r="C15">
+        <v>6</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>135</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B16">
         <v>351</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>404</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B17">
         <v>490</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
+      <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>117</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B18">
         <v>350</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>328</v>
       </c>
-      <c r="B19" t="n">
+      <c r="B19">
         <v>363</v>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
+      <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>287</v>
       </c>
-      <c r="B20" t="n">
+      <c r="B20">
         <v>191</v>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
+      <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>537</v>
       </c>
-      <c r="B21" t="n">
+      <c r="B21">
         <v>517</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
+      <c r="C21">
+        <v>6</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>537</v>
       </c>
-      <c r="B22" t="n">
+      <c r="B22">
         <v>517</v>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
+      <c r="C22">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>350</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B23">
         <v>306</v>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
+      <c r="C23">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>58</v>
       </c>
-      <c r="B24" t="n">
+      <c r="B24">
         <v>25</v>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
+      <c r="C24">
+        <v>6</v>
+      </c>
+      <c r="D24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>140</v>
       </c>
-      <c r="B25" t="n">
+      <c r="B25">
         <v>18</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
+      <c r="C25">
+        <v>6</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>18</v>
       </c>
-      <c r="B26" t="n">
+      <c r="B26">
         <v>140</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
+      <c r="C26">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>165</v>
       </c>
-      <c r="B27" t="n">
+      <c r="B27">
         <v>350</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
+      <c r="C27">
+        <v>6</v>
+      </c>
+      <c r="D27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>370</v>
       </c>
-      <c r="B28" t="n">
+      <c r="B28">
         <v>350</v>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
+      <c r="C28">
+        <v>6</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>56</v>
       </c>
-      <c r="B29" t="n">
+      <c r="B29">
         <v>25</v>
+      </c>
+      <c r="C29">
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed some railyway system logical issues (Added external riders).
Adjusted transport generation
</commit_message>
<xml_diff>
--- a/map/city/routes.xlsx
+++ b/map/city/routes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Unida\Documents\VSC\Python\EpidemicSimulation\map\city\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C87B59-CBA2-485D-8E76-543DEB4449BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D315B4-E40F-4381-8F67-7039D4EC4ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24300" yWindow="588" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -419,10 +419,10 @@
         <v>535</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -433,10 +433,10 @@
         <v>224</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -447,10 +447,10 @@
         <v>169</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -461,10 +461,10 @@
         <v>535</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -475,10 +475,10 @@
         <v>532</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -489,10 +489,10 @@
         <v>303</v>
       </c>
       <c r="C7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -503,10 +503,10 @@
         <v>111</v>
       </c>
       <c r="C8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -517,10 +517,10 @@
         <v>303</v>
       </c>
       <c r="C9">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -531,10 +531,10 @@
         <v>72</v>
       </c>
       <c r="C10">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -545,10 +545,10 @@
         <v>532</v>
       </c>
       <c r="C11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D11">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -559,10 +559,10 @@
         <v>365</v>
       </c>
       <c r="C12">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D12">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -573,10 +573,10 @@
         <v>537</v>
       </c>
       <c r="C13">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -587,10 +587,10 @@
         <v>285</v>
       </c>
       <c r="C14">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D14">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -601,10 +601,10 @@
         <v>537</v>
       </c>
       <c r="C15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D15">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -615,10 +615,10 @@
         <v>351</v>
       </c>
       <c r="C16">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D16">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -629,10 +629,10 @@
         <v>490</v>
       </c>
       <c r="C17">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D17">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -643,10 +643,10 @@
         <v>350</v>
       </c>
       <c r="C18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D18">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -657,10 +657,10 @@
         <v>363</v>
       </c>
       <c r="C19">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -671,10 +671,10 @@
         <v>191</v>
       </c>
       <c r="C20">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D20">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -685,10 +685,10 @@
         <v>517</v>
       </c>
       <c r="C21">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D21">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -699,10 +699,10 @@
         <v>517</v>
       </c>
       <c r="C22">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D22">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -713,10 +713,10 @@
         <v>306</v>
       </c>
       <c r="C23">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D23">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -727,10 +727,10 @@
         <v>25</v>
       </c>
       <c r="C24">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -741,10 +741,10 @@
         <v>18</v>
       </c>
       <c r="C25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D25">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -755,10 +755,10 @@
         <v>140</v>
       </c>
       <c r="C26">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D26">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -769,10 +769,10 @@
         <v>350</v>
       </c>
       <c r="C27">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -783,10 +783,10 @@
         <v>350</v>
       </c>
       <c r="C28">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D28">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -797,10 +797,10 @@
         <v>25</v>
       </c>
       <c r="C29">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated simulation scale for efficiency
</commit_message>
<xml_diff>
--- a/map/city/routes.xlsx
+++ b/map/city/routes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Unida\Documents\VSC\Python\EpidemicSimulation\map\city\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D315B4-E40F-4381-8F67-7039D4EC4ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D95B43B4-4DF5-48E8-90D1-AD66EDA94DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -419,10 +419,10 @@
         <v>535</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -433,10 +433,10 @@
         <v>224</v>
       </c>
       <c r="C3">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -447,10 +447,10 @@
         <v>169</v>
       </c>
       <c r="C4">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -461,10 +461,10 @@
         <v>535</v>
       </c>
       <c r="C5">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -475,10 +475,10 @@
         <v>532</v>
       </c>
       <c r="C6">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -489,10 +489,10 @@
         <v>303</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -503,10 +503,10 @@
         <v>111</v>
       </c>
       <c r="C8">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -517,10 +517,10 @@
         <v>303</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -531,10 +531,10 @@
         <v>72</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -545,10 +545,10 @@
         <v>532</v>
       </c>
       <c r="C11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -559,10 +559,10 @@
         <v>365</v>
       </c>
       <c r="C12">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -573,10 +573,10 @@
         <v>537</v>
       </c>
       <c r="C13">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -587,10 +587,10 @@
         <v>285</v>
       </c>
       <c r="C14">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D14">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -601,10 +601,10 @@
         <v>537</v>
       </c>
       <c r="C15">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D15">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -615,10 +615,10 @@
         <v>351</v>
       </c>
       <c r="C16">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -629,10 +629,10 @@
         <v>490</v>
       </c>
       <c r="C17">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D17">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -643,10 +643,10 @@
         <v>350</v>
       </c>
       <c r="C18">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D18">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -657,10 +657,10 @@
         <v>363</v>
       </c>
       <c r="C19">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -671,10 +671,10 @@
         <v>191</v>
       </c>
       <c r="C20">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D20">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -685,10 +685,10 @@
         <v>517</v>
       </c>
       <c r="C21">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D21">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -699,10 +699,10 @@
         <v>517</v>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D22">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -713,10 +713,10 @@
         <v>306</v>
       </c>
       <c r="C23">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -727,10 +727,10 @@
         <v>25</v>
       </c>
       <c r="C24">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D24">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -741,10 +741,10 @@
         <v>18</v>
       </c>
       <c r="C25">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D25">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -755,10 +755,10 @@
         <v>140</v>
       </c>
       <c r="C26">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D26">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -769,10 +769,10 @@
         <v>350</v>
       </c>
       <c r="C27">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D27">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -783,10 +783,10 @@
         <v>350</v>
       </c>
       <c r="C28">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D28">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -797,10 +797,10 @@
         <v>25</v>
       </c>
       <c r="C29">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D29">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed some bugs and implemented optimization for faster simulation speed
</commit_message>
<xml_diff>
--- a/map/city/routes.xlsx
+++ b/map/city/routes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Unida\Documents\VSC\Python\EpidemicSimulation\map\city\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AECF58-56C5-4557-9B50-9F149D89A4E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5933A12A-0854-4DCA-8472-D6B7F32380D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -395,9 +395,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -411,7 +411,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>23</v>
       </c>
@@ -425,7 +425,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>137</v>
       </c>
@@ -439,7 +439,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>109</v>
       </c>
@@ -453,7 +453,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>25</v>
       </c>
@@ -467,7 +467,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>28</v>
       </c>
@@ -481,7 +481,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>336</v>
       </c>
@@ -495,7 +495,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>46</v>
       </c>
@@ -509,7 +509,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>365</v>
       </c>
@@ -523,7 +523,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>137</v>
       </c>
@@ -537,7 +537,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>28</v>
       </c>
@@ -551,7 +551,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>491</v>
       </c>
@@ -565,7 +565,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>530</v>
       </c>
@@ -579,7 +579,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>191</v>
       </c>
@@ -593,7 +593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>233</v>
       </c>
@@ -607,7 +607,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>135</v>
       </c>
@@ -621,7 +621,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>404</v>
       </c>
@@ -635,7 +635,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>117</v>
       </c>
@@ -649,7 +649,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>328</v>
       </c>
@@ -663,7 +663,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>287</v>
       </c>
@@ -677,7 +677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>537</v>
       </c>
@@ -691,7 +691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>537</v>
       </c>
@@ -705,7 +705,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>350</v>
       </c>
@@ -719,7 +719,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>58</v>
       </c>
@@ -733,7 +733,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>140</v>
       </c>
@@ -747,7 +747,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>18</v>
       </c>
@@ -761,7 +761,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>165</v>
       </c>
@@ -775,7 +775,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>370</v>
       </c>
@@ -789,7 +789,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>56</v>
       </c>

</xml_diff>